<commit_message>
feat: suite E2E governance completa (API workflow) + fix rate limit 60/min + fix create_request .one() + users por role
</commit_message>
<xml_diff>
--- a/Requisito de Teste.xlsx
+++ b/Requisito de Teste.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\MasterData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7D9FD4F7-E351-434B-8946-45BD3CA8C135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8773C4C7-DE72-40EF-8D6D-BD6DCF9E832A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AAF02FDC-F2D0-468C-ABC8-C655C47A7C08}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="45">
   <si>
     <t>Grupo</t>
   </si>
@@ -45,6 +45,139 @@
   </si>
   <si>
     <t>Descrição Teste</t>
+  </si>
+  <si>
+    <t>Tenant</t>
+  </si>
+  <si>
+    <t>Criação de Tenant dedicado para o teste</t>
+  </si>
+  <si>
+    <t>Perfis de Acesso</t>
+  </si>
+  <si>
+    <t>Criação</t>
+  </si>
+  <si>
+    <t>Edição</t>
+  </si>
+  <si>
+    <t>Criar os Perfis de Acesso (ou utilizar o que o seed já cria)</t>
+  </si>
+  <si>
+    <t>Criar um novo tipo de Perfil de Acesso exclusivo para este tenant/test</t>
+  </si>
+  <si>
+    <t>Editar um perfil já existente</t>
+  </si>
+  <si>
+    <t>Gestão de Usuários</t>
+  </si>
+  <si>
+    <t>Criar 1 usuário para cada tipo de perfil:
+- Admin
+- Compras
+- Fiscal
+- MRP
+- Contabilidade
+- Cadastro
+- Solicitante</t>
+  </si>
+  <si>
+    <t>Modificar o nome de um usuário</t>
+  </si>
+  <si>
+    <t>Modificar a senha de um usuário e validar o acesso com a nova senha</t>
+  </si>
+  <si>
+    <t>Mudar o perfil de acesso e validar as permissões novas</t>
+  </si>
+  <si>
+    <t>Inativar um usuário e validar se o acesso é bloqueado</t>
+  </si>
+  <si>
+    <t>Solicitações</t>
+  </si>
+  <si>
+    <t>Link de Pesquisa</t>
+  </si>
+  <si>
+    <t>Validar se o item aparece ao efetuar a pesquisa</t>
+  </si>
+  <si>
+    <t>Validar se os detalhes do item abrem corretamente sem quebrar a tela</t>
+  </si>
+  <si>
+    <t>Botão "Não encontrei, criar solicitação" deverá direcionar para a Fase 1</t>
+  </si>
+  <si>
+    <t>Fase 1</t>
+  </si>
+  <si>
+    <t>Selecionar a urgência (criar uma solicitação para cada, para testar o indicador)</t>
+  </si>
+  <si>
+    <t>Botão "Próximo" direcionar para Fase 2</t>
+  </si>
+  <si>
+    <t>Fase 2</t>
+  </si>
+  <si>
+    <t>Botão "Voltar" direcionar para Link de Pesquisa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selecionar o PDM </t>
+  </si>
+  <si>
+    <t>Clicar em "Próximo" sem preencher os campos obrigatórios e validar que gerou mensagem de erro</t>
+  </si>
+  <si>
+    <t>Botão "Voltar" direcionar para Fase 1</t>
+  </si>
+  <si>
+    <t>Preencher campo a campo e confirmar o modal do "Preview da Descrição" vai atualizando a descrição e o avanço da %.</t>
+  </si>
+  <si>
+    <t>Botão "Próximo" direcionar para Fase 3</t>
+  </si>
+  <si>
+    <t>Inserir anexo</t>
+  </si>
+  <si>
+    <t>Fase 3</t>
+  </si>
+  <si>
+    <t>Botão "Voltar" direcionar para Fase 2</t>
+  </si>
+  <si>
+    <t>Botão "Próximo" direcionar para Fase 4</t>
+  </si>
+  <si>
+    <t>Fase 4</t>
+  </si>
+  <si>
+    <t>Botão "Voltar" direcionar para Fase 4</t>
+  </si>
+  <si>
+    <t>Botão "Finalizar Solicitação" deverá mostrar toast com o número da solicitação e direcionar para tela inicial.</t>
+  </si>
+  <si>
+    <t>Exportar</t>
+  </si>
+  <si>
+    <t>Utilizar a funcionalidade do botão "Exportar Excel" e validar se o arquivo abre com as informações.</t>
+  </si>
+  <si>
+    <t>Utilizar a funcionalidade do botão "Importação em Massa".</t>
+  </si>
+  <si>
+    <t>Baixar a planilha de template, abri-la e validar se está ok.</t>
+  </si>
+  <si>
+    <t>Verificar o botão Validar Planilha está ok.</t>
+  </si>
+  <si>
+    <t>Importação</t>
   </si>
 </sst>
 </file>
@@ -109,11 +242,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -449,218 +596,415 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DE74F8A-6022-4012-B7E5-B6B356C05C32}">
-  <dimension ref="B2:D41"/>
+  <dimension ref="B2:D45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="40.44140625" customWidth="1"/>
+    <col min="1" max="1" width="8.88671875" style="2"/>
+    <col min="2" max="2" width="19.77734375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="75.77734375" style="6" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="5" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
+      <c r="B3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
+      <c r="B4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
+      <c r="B5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-    </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
+      <c r="B6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="B7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
+      <c r="B8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
+      <c r="B9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
+      <c r="B10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
+      <c r="B11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
+      <c r="B12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
+      <c r="B13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-    </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
+      <c r="B14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B15" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
+      <c r="B16" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
+      <c r="B17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
+      <c r="B18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
+      <c r="B19" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
+      <c r="B20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
+      <c r="B21" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-    </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
+      <c r="B22" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B23" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-    </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
+      <c r="B24" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B25" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
+      <c r="B26" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
+      <c r="B27" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
+      <c r="B28" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
+      <c r="B29" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-    </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
+      <c r="B30" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="31" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B31" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B32" s="1"/>
-      <c r="C32" s="1"/>
-      <c r="D32" s="1"/>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="4"/>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B33" s="1"/>
-      <c r="C33" s="1"/>
-      <c r="D33" s="1"/>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="4"/>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B34" s="1"/>
-      <c r="C34" s="1"/>
-      <c r="D34" s="1"/>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="4"/>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B35" s="1"/>
-      <c r="C35" s="1"/>
-      <c r="D35" s="1"/>
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="4"/>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B36" s="1"/>
-      <c r="C36" s="1"/>
-      <c r="D36" s="1"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="4"/>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B37" s="1"/>
-      <c r="C37" s="1"/>
-      <c r="D37" s="1"/>
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="4"/>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B38" s="1"/>
-      <c r="C38" s="1"/>
-      <c r="D38" s="1"/>
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="4"/>
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B39" s="1"/>
-      <c r="C39" s="1"/>
-      <c r="D39" s="1"/>
+      <c r="B39" s="3"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="4"/>
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B40" s="1"/>
-      <c r="C40" s="1"/>
-      <c r="D40" s="1"/>
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="4"/>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B41" s="1"/>
-      <c r="C41" s="1"/>
-      <c r="D41" s="1"/>
+      <c r="B41" s="3"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="4"/>
+    </row>
+    <row r="42" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B42" s="3"/>
+      <c r="C42" s="3"/>
+      <c r="D42" s="4"/>
+    </row>
+    <row r="43" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B43" s="3"/>
+      <c r="C43" s="3"/>
+      <c r="D43" s="4"/>
+    </row>
+    <row r="44" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="4"/>
+    </row>
+    <row r="45" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>